<commit_message>
Complete regional model selections and extraction workflow guidance
</commit_message>
<xml_diff>
--- a/regions/EEZ_598/EEZ_598.xlsx
+++ b/regions/EEZ_598/EEZ_598.xlsx
@@ -435,240 +435,265 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<ns0:worksheet xmlns:ns0="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <ns0:sheetPr>
-    <ns0:outlinePr summaryBelow="1" summaryRight="1"/>
-    <ns0:pageSetUpPr fitToPage="1"/>
-  </ns0:sheetPr>
-  <ns0:sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <ns0:cols>
-    <ns0:col width="34" customWidth="1" min="1" max="1"/>
-    <ns0:col width="110" customWidth="1" min="2" max="2"/>
-    <ns0:col width="23" customWidth="1" min="3" max="3"/>
-    <ns0:col width="23" customWidth="1" min="4" max="4"/>
-    <ns0:col width="23" customWidth="1" min="5" max="5"/>
-    <ns0:col width="23" customWidth="1" min="6" max="6"/>
-    <ns0:col width="23" customWidth="1" min="7" max="7"/>
-    <ns0:col width="23" customWidth="1" min="8" max="8"/>
-  </ns0:cols>
-  <ns0:sheetData>
-    <ns0:row r="1">
-      <ns0:c r="A1" t="inlineStr">
-        <ns0:is>
-          <ns0:t>@table</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B1" t="inlineStr">
-        <ns0:is>
-          <ns0:t>Settings</ns0:t>
-        </ns0:is>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="2">
-      <ns0:c r="A2" s="1" t="inlineStr">
-        <ns0:is>
-          <ns0:t>field</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B2" s="1" t="inlineStr">
-        <ns0:is>
-          <ns0:t>value</ns0:t>
-        </ns0:is>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="3" ht="24" customHeight="1">
-      <ns0:c r="A3" s="2" t="inlineStr">
-        <ns0:is>
-          <ns0:t>unit_id</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B3" s="2" t="inlineStr">
-        <ns0:is>
-          <ns0:t>EEZ_598</ns0:t>
-        </ns0:is>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="4" ht="24" customHeight="1">
-      <ns0:c r="A4" s="2" t="inlineStr">
-        <ns0:is>
-          <ns0:t>region_name</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B4" s="2" t="inlineStr">
-        <ns0:is>
-          <ns0:t>Papua New Guinea</ns0:t>
-        </ns0:is>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="5" ht="24" customHeight="1">
-      <ns0:c r="A5" s="2" t="inlineStr">
-        <ns0:is>
-          <ns0:t>region_type</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B5" s="2" t="inlineStr">
-        <ns0:is>
-          <ns0:t>EEZ</ns0:t>
-        </ns0:is>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="6">
-      <ns0:c r="A6" s="2" t="inlineStr">
-        <ns0:is>
-          <ns0:t>selected_model_id</ns0:t>
-        </ns0:is>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="7">
-      <ns0:c r="A7" s="2" t="inlineStr">
-        <ns0:is>
-          <ns0:t>selection_rationale</ns0:t>
-        </ns0:is>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="8">
-      <ns0:c r="A8" s="2" t="inlineStr">
-        <ns0:is>
-          <ns0:t>model_path</ns0:t>
-        </ns0:is>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="9">
-      <ns0:c r="A9" s="2" t="inlineStr">
-        <ns0:is>
-          <ns0:t>results_model_id</ns0:t>
-        </ns0:is>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="10">
-      <ns0:c r="A10" s="2" t="inlineStr">
-        <ns0:is>
-          <ns0:t>results_model_sha256</ns0:t>
-        </ns0:is>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="11" ht="24" customHeight="1">
-      <ns0:c r="A11" s="2" t="inlineStr">
-        <ns0:is>
-          <ns0:t>selected_paper_ids</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B11" s="2" t="inlineStr"/>
-    </ns0:row>
-    <ns0:row r="12" ht="24" customHeight="1">
-      <ns0:c r="A12" s="2" t="inlineStr">
-        <ns0:is>
-          <ns0:t>production_eligible</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B12" t="b">
-        <ns0:v>0</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="13" ht="24" customHeight="1">
-      <ns0:c r="A13" s="2" t="inlineStr">
-        <ns0:is>
-          <ns0:t>catch_basis</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B13" s="2" t="inlineStr">
-        <ns0:is>
-          <ns0:t>landings</ns0:t>
-        </ns0:is>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="14" ht="24" customHeight="1">
-      <ns0:c r="A14" s="2" t="inlineStr">
-        <ns0:is>
-          <ns0:t>transfer_efficiency</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B14" s="3" t="n">
-        <ns0:v>0.1</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="15" ht="24" customHeight="1">
-      <ns0:c r="A15" s="2" t="inlineStr">
-        <ns0:is>
-          <ns0:t>taxon_detail_year</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B15" s="3" t="n">
-        <ns0:v>2019</ns0:v>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="16" ht="24" customHeight="1">
-      <ns0:c r="A16" s="2" t="inlineStr">
-        <ns0:is>
-          <ns0:t>source_note</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B16" s="2" t="inlineStr"/>
-    </ns0:row>
-    <ns0:row r="17" ht="24" customHeight="1">
-      <ns0:c r="A17" s="2" t="inlineStr">
-        <ns0:is>
-          <ns0:t>calculation_status</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B17" s="2" t="inlineStr">
-        <ns0:is>
-          <ns0:t>migrated saved results; unavailable methods retained</ns0:t>
-        </ns0:is>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="18" ht="24" customHeight="1">
-      <ns0:c r="A18" s="2" t="inlineStr">
-        <ns0:is>
-          <ns0:t>source_region_workbook</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B18" s="2" t="inlineStr">
-        <ns0:is>
-          <ns0:t>original_research_archive/legacy/data/EEZ_598/EEZ_598.xlsx</ns0:t>
-        </ns0:is>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="19" ht="24" customHeight="1">
-      <ns0:c r="A19" s="2" t="inlineStr">
-        <ns0:is>
-          <ns0:t>npp_policy</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B19" s="2" t="inlineStr">
-        <ns0:is>
-          <ns0:t>Annual observed support; unsupported years stay blank; no earliest-year proxy by default</ns0:t>
-        </ns0:is>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="20" ht="24" customHeight="1">
-      <ns0:c r="A20" s="2" t="inlineStr">
-        <ns0:is>
-          <ns0:t>calculation_input_sha256</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B20" s="2" t="inlineStr">
-        <ns0:is>
-          <ns0:t>2aac1fdf335fb5646e4c266484b0cd108a56a3c99229f03126a5ed675641f275</ns0:t>
-        </ns0:is>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="21" ht="24" customHeight="1">
-      <ns0:c r="A21" s="2" t="inlineStr">
-        <ns0:is>
-          <ns0:t>calculation_result_sha256</ns0:t>
-        </ns0:is>
-      </ns0:c>
-      <ns0:c r="B21" s="2" t="inlineStr">
-        <ns0:is>
-          <ns0:t>1c216aa2e3f67177d703bfc8c253f34ac21c8c86539d91ba0ca10a6e4a8e4311</ns0:t>
-        </ns0:is>
-      </ns0:c>
-    </ns0:row>
-    <ns0:row r="22"/>
-  </ns0:sheetData>
-  <ns0:pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</ns0:worksheet>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="110" customWidth="1" min="2" max="2"/>
+    <col width="23" customWidth="1" min="3" max="3"/>
+    <col width="23" customWidth="1" min="4" max="4"/>
+    <col width="23" customWidth="1" min="5" max="5"/>
+    <col width="23" customWidth="1" min="6" max="6"/>
+    <col width="23" customWidth="1" min="7" max="7"/>
+    <col width="23" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>@table</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Settings</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>field</t>
+        </is>
+      </c>
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t>value</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="24" customHeight="1">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>unit_id</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>EEZ_598</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="24" customHeight="1">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>region_name</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Papua New Guinea</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="24" customHeight="1">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>region_type</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>EEZ</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="24" customHeight="1">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>selected_model_id</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>941_20070101_WCPO_Warm_Pool_Option1_(mixed_periods)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="128" customHeight="1">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>selection_rationale</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>USER SELECTED 2026-09-28: WCP-2007 option 1 (D_fixed_M0) for HS_071, EEZ_941 and EEZ_598. Explicit experimental variant preserves juvenile other-mortality flows and changes Small BET P/B to 1.4129713563375232, EE to 0.7898725981469387; Small YFT P/B to 2.5304972811160384, EE to 0.8816702937266387. GE, TE and With Egestion all WARN; PP-budget checks OK, but strict mass balance remains false (adult BET residual 0.727940%). This is an adopted surrogate, not an author-confirmed correction or a region-specific native EwE model. Original source remains preserved. Griffiths 2019 source and pooled variant are retained for later investigation of failures, not selected.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="32" customHeight="1">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>model_path</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>models/941_20070101_WCPO_Warm_Pool_Option1_(mixed_periods)/941_20070101_WCPO_Warm_Pool_Option1_(mixed_periods).json</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="24" customHeight="1">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>results_model_id</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="24" customHeight="1">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>results_model_sha256</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="24" customHeight="1">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>selected_paper_ids</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="24" customHeight="1">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>production_eligible</t>
+        </is>
+      </c>
+      <c r="B12" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" ht="24" customHeight="1">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>catch_basis</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>landings</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="24" customHeight="1">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>transfer_efficiency</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="15" ht="24" customHeight="1">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>taxon_detail_year</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n">
+        <v>2019</v>
+      </c>
+    </row>
+    <row r="16" ht="24" customHeight="1">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>source_note</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="24" customHeight="1">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>calculation_status</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>selected; SPPR, matching and model PPR not yet calculated</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="24" customHeight="1">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>source_region_workbook</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>original_research_archive/legacy/data/EEZ_598/EEZ_598.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="24" customHeight="1">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>npp_policy</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>Annual observed support; unsupported years stay blank; no earliest-year proxy by default</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="24" customHeight="1">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>calculation_input_sha256</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>2aac1fdf335fb5646e4c266484b0cd108a56a3c99229f03126a5ed675641f275</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="24" customHeight="1">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>calculation_result_sha256</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>1c216aa2e3f67177d703bfc8c253f34ac21c8c86539d91ba0ca10a6e4a8e4311</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="96" customHeight="1">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>griffiths_later_investigation</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>USER REQUEST 2026-09-28: retain Griffiths et al. (2019) for later investigation across HS_071, EEZ_941 and EEZ_598. Understand why it fails before considering adoption. Original 46-group extraction is blocked by unknown two-pool routing. The authorized 45-group pooled experiment loads but GE, TE and With Egestion all FAIL. Investigate the Pomfret production/predation inconsistency, 22 printed catch-total versus fleet-sum conflicts, and routing/fishery-return and loader effects separately. No further parameter repair is authorized by this note.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23"/>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -76252,7 +76277,6 @@
       </c>
     </row>
     <row r="61">
-      <c r="A61" t="inlineStr"/>
       <c r="B61" t="inlineStr">
         <is>
           <t>all</t>
@@ -76495,7 +76519,6 @@
       </c>
     </row>
     <row r="62">
-      <c r="A62" t="inlineStr"/>
       <c r="B62" t="inlineStr">
         <is>
           <t>all</t>
@@ -76738,7 +76761,6 @@
       </c>
     </row>
     <row r="63">
-      <c r="A63" t="inlineStr"/>
       <c r="B63" t="inlineStr">
         <is>
           <t>all</t>
@@ -76981,7 +77003,6 @@
       </c>
     </row>
     <row r="64">
-      <c r="A64" t="inlineStr"/>
       <c r="B64" t="inlineStr">
         <is>
           <t>all</t>
@@ -77014,7 +77035,6 @@
       </c>
     </row>
     <row r="65">
-      <c r="A65" t="inlineStr"/>
       <c r="B65" t="inlineStr">
         <is>
           <t>all</t>
@@ -77047,7 +77067,6 @@
       </c>
     </row>
     <row r="66">
-      <c r="A66" t="inlineStr"/>
       <c r="B66" t="inlineStr">
         <is>
           <t>all</t>
@@ -77290,7 +77309,6 @@
       </c>
     </row>
     <row r="67">
-      <c r="A67" t="inlineStr"/>
       <c r="B67" t="inlineStr">
         <is>
           <t>all</t>
@@ -77533,7 +77551,6 @@
       </c>
     </row>
     <row r="68">
-      <c r="A68" t="inlineStr"/>
       <c r="B68" t="inlineStr">
         <is>
           <t>all</t>
@@ -77776,7 +77793,6 @@
       </c>
     </row>
     <row r="69">
-      <c r="A69" t="inlineStr"/>
       <c r="B69" t="inlineStr">
         <is>
           <t>all</t>
@@ -78019,7 +78035,6 @@
       </c>
     </row>
     <row r="70">
-      <c r="A70" t="inlineStr"/>
       <c r="B70" t="inlineStr">
         <is>
           <t>all</t>
@@ -78262,7 +78277,6 @@
       </c>
     </row>
     <row r="71">
-      <c r="A71" t="inlineStr"/>
       <c r="B71" t="inlineStr">
         <is>
           <t>all</t>
@@ -78505,7 +78519,6 @@
       </c>
     </row>
     <row r="72">
-      <c r="A72" t="inlineStr"/>
       <c r="B72" t="inlineStr">
         <is>
           <t>all</t>
@@ -78748,7 +78761,6 @@
       </c>
     </row>
     <row r="73">
-      <c r="A73" t="inlineStr"/>
       <c r="B73" t="inlineStr">
         <is>
           <t>all</t>
@@ -78991,7 +79003,6 @@
       </c>
     </row>
     <row r="74">
-      <c r="A74" t="inlineStr"/>
       <c r="B74" t="inlineStr">
         <is>
           <t>all</t>
@@ -79234,7 +79245,6 @@
       </c>
     </row>
     <row r="75">
-      <c r="A75" t="inlineStr"/>
       <c r="B75" t="inlineStr">
         <is>
           <t>all</t>
@@ -79267,7 +79277,6 @@
       </c>
     </row>
     <row r="76">
-      <c r="A76" t="inlineStr"/>
       <c r="B76" t="inlineStr">
         <is>
           <t>all</t>
@@ -79300,7 +79309,6 @@
       </c>
     </row>
     <row r="77">
-      <c r="A77" t="inlineStr"/>
       <c r="B77" t="inlineStr">
         <is>
           <t>all</t>
@@ -79543,7 +79551,6 @@
       </c>
     </row>
     <row r="78">
-      <c r="A78" t="inlineStr"/>
       <c r="B78" t="inlineStr">
         <is>
           <t>all</t>
@@ -79786,7 +79793,6 @@
       </c>
     </row>
     <row r="79">
-      <c r="A79" t="inlineStr"/>
       <c r="B79" t="inlineStr">
         <is>
           <t>all</t>
@@ -80029,7 +80035,6 @@
       </c>
     </row>
     <row r="80">
-      <c r="A80" t="inlineStr"/>
       <c r="B80" t="inlineStr">
         <is>
           <t>all</t>
@@ -80272,7 +80277,6 @@
       </c>
     </row>
     <row r="81">
-      <c r="A81" t="inlineStr"/>
       <c r="B81" t="inlineStr">
         <is>
           <t>all</t>
@@ -80515,7 +80519,6 @@
       </c>
     </row>
     <row r="82">
-      <c r="A82" t="inlineStr"/>
       <c r="B82" t="inlineStr">
         <is>
           <t>all</t>
@@ -80758,7 +80761,6 @@
       </c>
     </row>
     <row r="83">
-      <c r="A83" t="inlineStr"/>
       <c r="B83" t="inlineStr">
         <is>
           <t>all</t>
@@ -81001,7 +81003,6 @@
       </c>
     </row>
     <row r="84">
-      <c r="A84" t="inlineStr"/>
       <c r="B84" t="inlineStr">
         <is>
           <t>all</t>
@@ -81244,7 +81245,6 @@
       </c>
     </row>
     <row r="85">
-      <c r="A85" t="inlineStr"/>
       <c r="B85" t="inlineStr">
         <is>
           <t>all</t>
@@ -81487,7 +81487,6 @@
       </c>
     </row>
     <row r="86">
-      <c r="A86" t="inlineStr"/>
       <c r="B86" t="inlineStr">
         <is>
           <t>all</t>
@@ -81520,7 +81519,6 @@
       </c>
     </row>
     <row r="87">
-      <c r="A87" t="inlineStr"/>
       <c r="B87" t="inlineStr">
         <is>
           <t>all</t>
@@ -81553,7 +81551,6 @@
       </c>
     </row>
     <row r="88">
-      <c r="A88" t="inlineStr"/>
       <c r="B88" t="inlineStr">
         <is>
           <t>all</t>
@@ -81796,7 +81793,6 @@
       </c>
     </row>
     <row r="89">
-      <c r="A89" t="inlineStr"/>
       <c r="B89" t="inlineStr">
         <is>
           <t>all</t>
@@ -82039,7 +82035,6 @@
       </c>
     </row>
     <row r="90">
-      <c r="A90" t="inlineStr"/>
       <c r="B90" t="inlineStr">
         <is>
           <t>all</t>
@@ -82282,7 +82277,6 @@
       </c>
     </row>
     <row r="91">
-      <c r="A91" t="inlineStr"/>
       <c r="B91" t="inlineStr">
         <is>
           <t>all</t>
@@ -82525,7 +82519,6 @@
       </c>
     </row>
     <row r="92">
-      <c r="A92" t="inlineStr"/>
       <c r="B92" t="inlineStr">
         <is>
           <t>all</t>
@@ -82768,7 +82761,6 @@
       </c>
     </row>
     <row r="93">
-      <c r="A93" t="inlineStr"/>
       <c r="B93" t="inlineStr">
         <is>
           <t>all</t>
@@ -87425,7 +87417,6 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr"/>
       <c r="B3" t="inlineStr">
         <is>
           <t>all</t>
@@ -87519,7 +87510,6 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr"/>
       <c r="B4" t="inlineStr">
         <is>
           <t>all</t>
@@ -87598,7 +87588,6 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr"/>
       <c r="B5" t="inlineStr">
         <is>
           <t>all</t>
@@ -87677,7 +87666,6 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr"/>
       <c r="B6" t="inlineStr">
         <is>
           <t>all</t>
@@ -87756,7 +87744,6 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr"/>
       <c r="B7" t="inlineStr">
         <is>
           <t>all</t>
@@ -87835,7 +87822,6 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr"/>
       <c r="B8" t="inlineStr">
         <is>
           <t>all</t>
@@ -87929,7 +87915,6 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr"/>
       <c r="B9" t="inlineStr">
         <is>
           <t>all</t>
@@ -88023,7 +88008,6 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr"/>
       <c r="B10" t="inlineStr">
         <is>
           <t>all</t>
@@ -88102,7 +88086,6 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr"/>
       <c r="B11" t="inlineStr">
         <is>
           <t>all</t>
@@ -88181,7 +88164,6 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr"/>
       <c r="B12" t="inlineStr">
         <is>
           <t>all</t>
@@ -88260,7 +88242,6 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr"/>
       <c r="B13" t="inlineStr">
         <is>
           <t>all</t>
@@ -88339,7 +88320,6 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr"/>
       <c r="B14" t="inlineStr">
         <is>
           <t>all</t>
@@ -88433,7 +88413,6 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr"/>
       <c r="B15" t="inlineStr">
         <is>
           <t>all</t>
@@ -88527,7 +88506,6 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr"/>
       <c r="B16" t="inlineStr">
         <is>
           <t>all</t>
@@ -88606,7 +88584,6 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr"/>
       <c r="B17" t="inlineStr">
         <is>
           <t>all</t>
@@ -88685,7 +88662,6 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr"/>
       <c r="B18" t="inlineStr">
         <is>
           <t>all</t>
@@ -88764,7 +88740,6 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" t="inlineStr"/>
       <c r="B19" t="inlineStr">
         <is>
           <t>all</t>
@@ -88843,7 +88818,6 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" t="inlineStr"/>
       <c r="B20" t="inlineStr">
         <is>
           <t>all</t>
@@ -88937,7 +88911,6 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" t="inlineStr"/>
       <c r="B21" t="inlineStr">
         <is>
           <t>all</t>
@@ -89031,7 +89004,6 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" t="inlineStr"/>
       <c r="B22" t="inlineStr">
         <is>
           <t>all</t>
@@ -89110,7 +89082,6 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" t="inlineStr"/>
       <c r="B23" t="inlineStr">
         <is>
           <t>all</t>
@@ -89189,7 +89160,6 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" t="inlineStr"/>
       <c r="B24" t="inlineStr">
         <is>
           <t>all</t>
@@ -89268,7 +89238,6 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" t="inlineStr"/>
       <c r="B25" t="inlineStr">
         <is>
           <t>all</t>
@@ -89347,7 +89316,6 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" t="inlineStr"/>
       <c r="B26" t="inlineStr">
         <is>
           <t>all</t>
@@ -89441,7 +89409,6 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" t="inlineStr"/>
       <c r="B27" t="inlineStr">
         <is>
           <t>all</t>
@@ -89535,7 +89502,6 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" t="inlineStr"/>
       <c r="B28" t="inlineStr">
         <is>
           <t>all</t>
@@ -89614,7 +89580,6 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" t="inlineStr"/>
       <c r="B29" t="inlineStr">
         <is>
           <t>all</t>
@@ -89693,7 +89658,6 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" t="inlineStr"/>
       <c r="B30" t="inlineStr">
         <is>
           <t>all</t>
@@ -89772,7 +89736,6 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" t="inlineStr"/>
       <c r="B31" t="inlineStr">
         <is>
           <t>all</t>
@@ -89851,7 +89814,6 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" t="inlineStr"/>
       <c r="B32" t="inlineStr">
         <is>
           <t>all</t>
@@ -89945,7 +89907,6 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" t="inlineStr"/>
       <c r="B33" t="inlineStr">
         <is>
           <t>all</t>
@@ -90039,7 +90000,6 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" t="inlineStr"/>
       <c r="B34" t="inlineStr">
         <is>
           <t>all</t>
@@ -90118,7 +90078,6 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" t="inlineStr"/>
       <c r="B35" t="inlineStr">
         <is>
           <t>all</t>
@@ -90197,7 +90156,6 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" t="inlineStr"/>
       <c r="B36" t="inlineStr">
         <is>
           <t>all</t>
@@ -90276,7 +90234,6 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" t="inlineStr"/>
       <c r="B37" t="inlineStr">
         <is>
           <t>all</t>
@@ -90355,7 +90312,6 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" t="inlineStr"/>
       <c r="B38" t="inlineStr">
         <is>
           <t>all</t>
@@ -90449,7 +90405,6 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" t="inlineStr"/>
       <c r="B39" t="inlineStr">
         <is>
           <t>all</t>
@@ -90543,7 +90498,6 @@
       </c>
     </row>
     <row r="40">
-      <c r="A40" t="inlineStr"/>
       <c r="B40" t="inlineStr">
         <is>
           <t>all</t>
@@ -90622,7 +90576,6 @@
       </c>
     </row>
     <row r="41">
-      <c r="A41" t="inlineStr"/>
       <c r="B41" t="inlineStr">
         <is>
           <t>all</t>
@@ -90701,7 +90654,6 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" t="inlineStr"/>
       <c r="B42" t="inlineStr">
         <is>
           <t>all</t>
@@ -90780,7 +90732,6 @@
       </c>
     </row>
     <row r="43">
-      <c r="A43" t="inlineStr"/>
       <c r="B43" t="inlineStr">
         <is>
           <t>all</t>
@@ -90859,7 +90810,6 @@
       </c>
     </row>
     <row r="44">
-      <c r="A44" t="inlineStr"/>
       <c r="B44" t="inlineStr">
         <is>
           <t>all</t>
@@ -90953,7 +90903,6 @@
       </c>
     </row>
     <row r="45">
-      <c r="A45" t="inlineStr"/>
       <c r="B45" t="inlineStr">
         <is>
           <t>all</t>
@@ -91047,7 +90996,6 @@
       </c>
     </row>
     <row r="46">
-      <c r="A46" t="inlineStr"/>
       <c r="B46" t="inlineStr">
         <is>
           <t>all</t>
@@ -91126,7 +91074,6 @@
       </c>
     </row>
     <row r="47">
-      <c r="A47" t="inlineStr"/>
       <c r="B47" t="inlineStr">
         <is>
           <t>all</t>
@@ -91205,7 +91152,6 @@
       </c>
     </row>
     <row r="48">
-      <c r="A48" t="inlineStr"/>
       <c r="B48" t="inlineStr">
         <is>
           <t>all</t>
@@ -91284,7 +91230,6 @@
       </c>
     </row>
     <row r="49">
-      <c r="A49" t="inlineStr"/>
       <c r="B49" t="inlineStr">
         <is>
           <t>all</t>
@@ -91363,7 +91308,6 @@
       </c>
     </row>
     <row r="50">
-      <c r="A50" t="inlineStr"/>
       <c r="B50" t="inlineStr">
         <is>
           <t>all</t>
@@ -91457,7 +91401,6 @@
       </c>
     </row>
     <row r="51">
-      <c r="A51" t="inlineStr"/>
       <c r="B51" t="inlineStr">
         <is>
           <t>all</t>
@@ -91551,7 +91494,6 @@
       </c>
     </row>
     <row r="52">
-      <c r="A52" t="inlineStr"/>
       <c r="B52" t="inlineStr">
         <is>
           <t>all</t>
@@ -91630,7 +91572,6 @@
       </c>
     </row>
     <row r="53">
-      <c r="A53" t="inlineStr"/>
       <c r="B53" t="inlineStr">
         <is>
           <t>all</t>
@@ -91709,7 +91650,6 @@
       </c>
     </row>
     <row r="54">
-      <c r="A54" t="inlineStr"/>
       <c r="B54" t="inlineStr">
         <is>
           <t>all</t>
@@ -91788,7 +91728,6 @@
       </c>
     </row>
     <row r="55">
-      <c r="A55" t="inlineStr"/>
       <c r="B55" t="inlineStr">
         <is>
           <t>all</t>
@@ -91867,7 +91806,6 @@
       </c>
     </row>
     <row r="56">
-      <c r="A56" t="inlineStr"/>
       <c r="B56" t="inlineStr">
         <is>
           <t>all</t>

</xml_diff>